<commit_message>
docs: add Batch 3 delivery, operations, validation and customer documents
Scrum plan with roles, cadence, sprints to a January 2027 closed beta and
a cut line; product backlog of 43 user stories; SRE handbook with SLOs,
alerting, on-call, nine runbooks, backup and migration plan; validation
plan with eight hypotheses, experiments and decision rules; beta help
centre with seventeen articles.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KC7q2XdCVxuwsART7HEcsQ
</commit_message>
<xml_diff>
--- a/docs/registers/beatmind-registers.xlsx
+++ b/docs/registers/beatmind-registers.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entitlements" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12736,4 +12737,1786 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>epic_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>acceptance_criteria</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>points</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>linked</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>target_sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>US-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Foundations: repo, CI, environments, observability</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>As a developer, I want a monorepo with Java, Python and web modules building in CI, so that every change is tested</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CI runs unit tests, scans and RTM check on every pull request; main is protected</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>REQ-SEC-12</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>US-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Foundations: repo, CI, environments, observability</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>As a developer, I want Docker Compose for local development with a CPU model stub, so that I can work without a GPU</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>`docker compose up` starts web, API, Postgres, Valkey, MinIO and stub worker; README documents it</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>US-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Foundations: repo, CI, environments, observability</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>As an operator, I want staging and production environments defined in OpenTofu, so that environments are reproducible</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Plan and apply succeed from CI; secrets from vault</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>ADR-006; ADR-012</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>US-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Foundations: repo, CI, environments, observability</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>As an operator, I want OpenTelemetry traces, metrics and logs with dashboards, so that I can see SLOs</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Dashboards for latency, errors, queue depth, GPU use, cost per song</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>REQ-NFR-07</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>US-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Generation pipeline</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>As the team, I want ACE-Step 1.5 benchmarked on a rented GPU, so that we know real time and cost per take</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Report with seconds per take, VRAM, cost per take for 3 GPU types; licence file archived</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>A-025; C-02</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>US-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Lyrics and languages</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>As the team, I want a Hindi and Hinglish quality spike, so that we know if the beachhead language works</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>20 prompts per language generated and scored by 3 native speakers; go or fallback decision</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>A-021; RISK-003</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>US-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>EP-12</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Validation and growth (waitlist, interviews, listening tests)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>As the founder, I want a waitlist page with local prices shown, so that we measure interest and price response</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Page live in English and Hindi; sign-ups stored with consent; price variant recorded</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>H-001; H-004</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>US-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EP-12</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Validation and growth (waitlist, interviews, listening tests)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>As the founder, I want 20 creator interviews done with a script, so that demand hypotheses are tested</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Interview notes in repository; synthesis against H-001 to H-005</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>DEC-012</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>US-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Identity and accounts</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want to sign in with Google or an email code, so that I can start quickly</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Sign-in works; sessions secure per REQ-SEC-01; 18+ check at sign-up</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-53; REQ-SEC-01</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>US-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Identity and accounts</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want to choose English or Hindi, so that the app speaks my language</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Locale switch persists; all MVP strings in both languages</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-16; REQ-NFR-09</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>US-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Identity and accounts</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want to export or delete my data, so that I control my information</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Export JSON plus files; deletion per DPIA section 6</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>REQ-NFR-05</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>US-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Generation pipeline</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want to describe a vibe and get two takes, so that I get music for my video</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>API-001 and API-002 with SSE; two takes delivered; p95 under 60 s in staging</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-01; REQ-F-05</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>US-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Generation pipeline</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>As the system, I want a durable Postgres job queue with retries and dead-letter, so that jobs survive restarts</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Jobs claimed with SKIP LOCKED; retry with backoff; dead-letter visible in admin</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>ADR-005</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>US-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Generation pipeline</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want to see my queue position and wait time, so that I know when my song is ready</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Live region announces status; estimate within ±30%</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>UX-A11Y-15</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>US-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Generation pipeline</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>As a producer, I want Beat mode with genre, BPM, key and instruments, so that I can make instrumentals</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Validation per REQ-F-04; tempo check runs on output</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-04</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>US-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Generation pipeline</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>As the system, I want a Lyria fallback with a daily spend cap, so that paid users still get songs when GPUs are busy</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Fallback used only when routed; cap enforced; cost logged</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>ADR-007; REQ-SEC-09</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>US-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Lyrics and languages</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>As an artist, I want to paste lyrics in Hindi, Hinglish or English, so that my words become a song</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Grapheme counting; NFC; language tag stored; custom mode works</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-02; REQ-F-08</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>US-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Lyrics and languages</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want the AI to write lyrics from a topic and mood, so that I can make a song without writing</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Sectioned lyrics in chosen language; moderation applied</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-03</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>US-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Provenance, labelling and certificates</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>As the system, I want every event written to a hash-chained ledger, so that provenance is provable</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Chain verification test passes; tamper test fails as expected</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-31; REQ-SEC-07</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>US-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Provenance, labelling and certificates</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want my downloads labelled and watermarked with content credentials, so that they meet AI rules</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>AI label metadata, valid C2PA manifest, detectable watermark on every export</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-30; COMP-IN-02</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>US-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Provenance, labelling and certificates</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>As anyone, I want to verify a file or certificate, so that I can check its origin</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Verify page with rate limits and coarse anonymous answers</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-32; REQ-SEC-10</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>US-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Library, player and sharing</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want a library of my songs and takes, so that I can find my work</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>List, search (Unicode-aware), rename, delete</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-12</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>US-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Library, player and sharing</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want an accessible player that shows lyrics and the AI label, so that everyone can use it</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard operable; ARIA; lyrics shown; label visible</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-33; UX-A11Y-01 to 03</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>US-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Library, player and sharing</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want to share a private link or public page, so that others can hear my song</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Revocable share tokens; public page with moderation of title and lyrics</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-13; REQ-SEC-03</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>US-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Rights, quotas and downloads</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>As a free user, I want to mark up to 5 songs a month for commercial use, so that I can use them in videos</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Quota enforced; certificate issued; attribution text provided</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-21</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>US-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Rights, quotas and downloads</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want to download MP3 (and WAV when paid), so that I can use my song</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Signed URLs 15 min; formats by plan per entitlement matrix</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-20; REQ-F-23</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>US-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Rights, quotas and downloads</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want failed or withheld takes refunded, so that I never pay for nothing</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Automatic refund with ledger entry</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-56</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>US-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>EP-08</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Safety and moderation</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>As the platform, I want prompts and lyrics moderated in Hindi, Hinglish and English, so that harmful content is blocked</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Red-team set passes; Unicode corpus passes; reasons shown</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-50; REQ-F-51; REQ-SEC-04</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>US-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>EP-08</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Safety and moderation</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>As the platform, I want generated audio screened for similarity, so that near-copies are withheld</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Screen runs on every take; withheld takes logged and refunded</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-52</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>US-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>EP-08</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Safety and moderation</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>As the platform, I want bot defence and caps, so that free generation is not abused</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Turnstile; daily caps; concurrency limits; velocity rules</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-55; REQ-SEC-09</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>US-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>EP-09</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Admin and takedowns</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>As an admin, I want a console for users, caps and the moderation queue, so that I can run the beta</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Role-gated; MFA required; every action audited</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>FEAT-18; REQ-SEC-06</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>US-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>EP-09</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Admin and takedowns</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>As an admin, I want takedown and appeal workflows with deadline timers, so that we meet the 3-hour rule</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Orders path tested end to end; appeals queue works</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-54; REQ-F-59</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>US-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>EP-10</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Payments and pricing</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want to see prices in my currency for my country, so that the price is fair where I live</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Price bands applied by billing country</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-40; REQ-F-41</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>US-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>EP-10</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Payments and pricing</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>As an Indian user, I want to pay by UPI, card or net banking, so that I can subscribe</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Razorpay test and live mode; webhooks verified</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-42; REQ-SEC-08</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>US-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>EP-10</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Payments and pricing</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>As an international user, I want to pay through a merchant of record, so that taxes are handled</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Provider checkout; webhooks verified</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>ADR-009</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>US-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>EP-10</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Payments and pricing</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>As a paid user, I want ownership of songs I create, with a certificate, so that I can use them anywhere</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>user_owned state; certificate; vesting on settlement; chargeback rule</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-22; REQ-F-57</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>US-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>EP-10</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Payments and pricing</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want to cancel online easily and keep my owned songs, so that I trust the service</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Three-step cancel; downloads still available</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-43; REQ-F-58</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>US-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>EP-11</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Editor and stems</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>As a creator, I want to extend, trim, fade and regenerate a section, so that I can fix a take</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>New version per edit; seam test passes</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-10; REQ-F-11</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>US-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>EP-11</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Editor and stems</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>As a producer, I want four separated stems, so that I can mix my song</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Demucs stems; sum test; SDR reported</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>REQ-F-23</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>US-040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>EP-12</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Validation and growth (waitlist, interviews, listening tests)</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>As the team, I want G1 listening tests run for Hindi, Hinglish and English, so that we know which languages launch</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>30 listeners per language; results against pass mark</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>PRD 12</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>US-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>EP-12</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Validation and growth (waitlist, interviews, listening tests)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>As the founder, I want an investor demo script and recording, so that fundraising can start</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Five-minute demo of the beta flow on staging</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>A-003</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>US-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Foundations: repo, CI, environments, observability</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>As the team, I want a load test and a security baseline scan before beta, so that gate G2 is met</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>k6 at 2x beta peak; ZAP baseline; findings triaged</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>REQ-NFR-01; REQ-SEC-12</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>US-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Foundations: repo, CI, environments, observability</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>As the team, I want accessibility checks in CI and a manual screen-reader pass, so that WCAG 2.2 AA holds</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>axe-core in CI; manual pass recorded</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>REQ-NFR-08</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>SPRINT-04</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record DEC-027, open-model approach for the beta (Q-F04)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KC7q2XdCVxuwsART7HEcsQ
</commit_message>
<xml_diff>
--- a/docs/registers/beatmind-registers.xlsx
+++ b/docs/registers/beatmind-registers.xlsx
@@ -652,12 +652,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Source-stated</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Default for Q-F04</t>
+          <t>Founder answer</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Confirmed by founder 2026-10-29 (DEC-027)</t>
         </is>
       </c>
     </row>

</xml_diff>